<commit_message>
Add in the gain
</commit_message>
<xml_diff>
--- a/Acoustics/Exam_1_Folder/high_pass_resistor.xlsx
+++ b/Acoustics/Exam_1_Folder/high_pass_resistor.xlsx
@@ -1,17 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_1A0AB6144E82C05A6A46777B7253018143AC288F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CADF90D3-C8E1-4F32-AB31-53E9CCE64C00}"/>
+  <bookViews>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="13372" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>DataPtNum</t>
   </si>
@@ -27,21 +44,29 @@
   <si>
     <t>phase</t>
   </si>
+  <si>
+    <t>Gain (|Vout/Vin|)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -69,9 +94,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,15 +436,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E50"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F50"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11" customWidth="1"/>
     <col min="3" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="18.07421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -434,8 +461,11 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -451,8 +481,12 @@
       <c r="E2">
         <v>154</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="2">
+        <f>D2/C2</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -468,8 +502,12 @@
       <c r="E3">
         <v>86.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" s="2">
+        <f t="shared" ref="F3:F50" si="0">D3/C3</f>
+        <v>3.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -480,13 +518,17 @@
         <v>10</v>
       </c>
       <c r="D4">
-        <v>0.032</v>
+        <v>3.2000000000000001E-2</v>
       </c>
       <c r="E4">
         <v>168</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="2">
+        <f t="shared" si="0"/>
+        <v>3.2000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -497,13 +539,17 @@
         <v>10</v>
       </c>
       <c r="D5">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="E5">
         <v>92.9</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="2">
+        <f t="shared" si="0"/>
+        <v>3.4000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -514,13 +560,17 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>0.035</v>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="E6">
         <v>168</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
+        <v>3.5000000000000005E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>6</v>
       </c>
@@ -531,13 +581,17 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>0.034</v>
+        <v>3.4000000000000002E-2</v>
       </c>
       <c r="E7">
         <v>115</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="2">
+        <f t="shared" si="0"/>
+        <v>3.4000000000000002E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>7</v>
       </c>
@@ -548,13 +602,17 @@
         <v>10</v>
       </c>
       <c r="D8">
-        <v>0.038</v>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="E8">
         <v>115</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>3.8E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>8</v>
       </c>
@@ -570,8 +628,12 @@
       <c r="E9">
         <v>101</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>9</v>
       </c>
@@ -582,13 +644,17 @@
         <v>10</v>
       </c>
       <c r="D10">
-        <v>0.043</v>
+        <v>4.2999999999999997E-2</v>
       </c>
       <c r="E10">
         <v>121</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>4.3E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>10</v>
       </c>
@@ -599,13 +665,17 @@
         <v>10</v>
       </c>
       <c r="D11">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="E11">
         <v>120</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>4.8000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>11</v>
       </c>
@@ -616,13 +686,17 @@
         <v>10</v>
       </c>
       <c r="D12">
-        <v>0.048</v>
+        <v>4.8000000000000001E-2</v>
       </c>
       <c r="E12">
         <v>118</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="2">
+        <f t="shared" si="0"/>
+        <v>4.8000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>12</v>
       </c>
@@ -633,13 +707,17 @@
         <v>10</v>
       </c>
       <c r="D13">
-        <v>0.051</v>
+        <v>5.0999999999999997E-2</v>
       </c>
       <c r="E13">
         <v>128</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="2">
+        <f t="shared" si="0"/>
+        <v>5.0999999999999995E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>13</v>
       </c>
@@ -647,16 +725,20 @@
         <v>100</v>
       </c>
       <c r="C14">
-        <v>9.8</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="D14">
-        <v>0.053</v>
+        <v>5.2999999999999999E-2</v>
       </c>
       <c r="E14">
         <v>123</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="2">
+        <f t="shared" si="0"/>
+        <v>5.4081632653061222E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>14</v>
       </c>
@@ -664,7 +746,7 @@
         <v>150</v>
       </c>
       <c r="C15">
-        <v>9.2</v>
+        <v>9.1999999999999993</v>
       </c>
       <c r="D15">
         <v>0.08</v>
@@ -672,8 +754,12 @@
       <c r="E15">
         <v>128</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="2">
+        <f t="shared" si="0"/>
+        <v>8.6956521739130436E-3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>15</v>
       </c>
@@ -681,7 +767,7 @@
         <v>200</v>
       </c>
       <c r="C16">
-        <v>8.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="D16">
         <v>0.1</v>
@@ -689,8 +775,12 @@
       <c r="E16">
         <v>121</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="2">
+        <f t="shared" si="0"/>
+        <v>1.1363636363636364E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A17">
         <v>16</v>
       </c>
@@ -701,13 +791,17 @@
         <v>8</v>
       </c>
       <c r="D17">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E17">
         <v>130</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="2">
+        <f t="shared" si="0"/>
+        <v>1.7500000000000002E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A18">
         <v>17</v>
       </c>
@@ -718,13 +812,17 @@
         <v>7.6</v>
       </c>
       <c r="D18">
-        <v>0.172</v>
+        <v>0.17199999999999999</v>
       </c>
       <c r="E18">
         <v>136</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="2">
+        <f t="shared" si="0"/>
+        <v>2.2631578947368419E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A19">
         <v>18</v>
       </c>
@@ -740,8 +838,12 @@
       <c r="E19">
         <v>139</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="2">
+        <f t="shared" si="0"/>
+        <v>3.0303030303030307E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20">
         <v>19</v>
       </c>
@@ -757,8 +859,12 @@
       <c r="E20">
         <v>134</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="2">
+        <f t="shared" si="0"/>
+        <v>3.8709677419354833E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A21">
         <v>20</v>
       </c>
@@ -774,8 +880,12 @@
       <c r="E21">
         <v>132</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="2">
+        <f t="shared" si="0"/>
+        <v>4.6551724137931037E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A22">
         <v>21</v>
       </c>
@@ -786,13 +896,17 @@
         <v>5.4</v>
       </c>
       <c r="D22">
-        <v>0.296</v>
+        <v>0.29599999999999999</v>
       </c>
       <c r="E22">
         <v>133</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F22" s="2">
+        <f t="shared" si="0"/>
+        <v>5.4814814814814809E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A23">
         <v>22</v>
       </c>
@@ -808,8 +922,12 @@
       <c r="E23">
         <v>140</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" s="2">
+        <f t="shared" si="0"/>
+        <v>6.4000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A24">
         <v>23</v>
       </c>
@@ -817,16 +935,20 @@
         <v>600</v>
       </c>
       <c r="C24">
-        <v>4.48</v>
+        <v>4.4800000000000004</v>
       </c>
       <c r="D24">
-        <v>0.344</v>
+        <v>0.34399999999999997</v>
       </c>
       <c r="E24">
         <v>136</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F24" s="2">
+        <f t="shared" si="0"/>
+        <v>7.6785714285714277E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A25">
         <v>24</v>
       </c>
@@ -842,8 +964,12 @@
       <c r="E25">
         <v>124</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F25" s="2">
+        <f t="shared" si="0"/>
+        <v>8.8679245283018862E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A26">
         <v>25</v>
       </c>
@@ -859,8 +985,12 @@
       <c r="E26">
         <v>135</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F26" s="2">
+        <f t="shared" si="0"/>
+        <v>0.10204081632653061</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A27">
         <v>26</v>
       </c>
@@ -871,13 +1001,17 @@
         <v>3.68</v>
       </c>
       <c r="D27">
-        <v>0.424</v>
+        <v>0.42399999999999999</v>
       </c>
       <c r="E27">
         <v>147</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F27" s="2">
+        <f t="shared" si="0"/>
+        <v>0.11521739130434781</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A28">
         <v>27</v>
       </c>
@@ -893,8 +1027,12 @@
       <c r="E28">
         <v>122</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F28" s="2">
+        <f t="shared" si="0"/>
+        <v>0.12790697674418605</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A29">
         <v>28</v>
       </c>
@@ -905,13 +1043,17 @@
         <v>3.28</v>
       </c>
       <c r="D29">
-        <v>0.464</v>
+        <v>0.46400000000000002</v>
       </c>
       <c r="E29">
         <v>121</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F29" s="2">
+        <f t="shared" si="0"/>
+        <v>0.14146341463414636</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A30">
         <v>29</v>
       </c>
@@ -922,13 +1064,17 @@
         <v>3.12</v>
       </c>
       <c r="D30">
-        <v>0.488</v>
+        <v>0.48799999999999999</v>
       </c>
       <c r="E30">
         <v>121</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F30" s="2">
+        <f t="shared" si="0"/>
+        <v>0.15641025641025641</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A31">
         <v>30</v>
       </c>
@@ -944,8 +1090,12 @@
       <c r="E31">
         <v>125</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F31" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16891891891891891</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A32">
         <v>31</v>
       </c>
@@ -956,13 +1106,17 @@
         <v>2.8</v>
       </c>
       <c r="D32">
-        <v>0.512</v>
+        <v>0.51200000000000001</v>
       </c>
       <c r="E32">
         <v>111</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F32" s="2">
+        <f t="shared" si="0"/>
+        <v>0.18285714285714288</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A33">
         <v>32</v>
       </c>
@@ -973,13 +1127,17 @@
         <v>1.84</v>
       </c>
       <c r="D33">
-        <v>0.616</v>
+        <v>0.61599999999999999</v>
       </c>
       <c r="E33">
         <v>99</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F33" s="2">
+        <f t="shared" si="0"/>
+        <v>0.33478260869565213</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A34">
         <v>33</v>
       </c>
@@ -990,13 +1148,17 @@
         <v>1.52</v>
       </c>
       <c r="D34">
-        <v>0.664</v>
+        <v>0.66400000000000003</v>
       </c>
       <c r="E34">
-        <v>75.6</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>75.599999999999994</v>
+      </c>
+      <c r="F34" s="2">
+        <f t="shared" si="0"/>
+        <v>0.43684210526315792</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1007,13 +1169,17 @@
         <v>1.36</v>
       </c>
       <c r="D35">
-        <v>0.696</v>
+        <v>0.69599999999999995</v>
       </c>
       <c r="E35">
         <v>76.5</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" s="2">
+        <f t="shared" si="0"/>
+        <v>0.5117647058823529</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1024,13 +1190,17 @@
         <v>1.2</v>
       </c>
       <c r="D36">
-        <v>0.712</v>
+        <v>0.71199999999999997</v>
       </c>
       <c r="E36">
         <v>47.6</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F36" s="2">
+        <f t="shared" si="0"/>
+        <v>0.59333333333333338</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1046,8 +1216,12 @@
       <c r="E37">
         <v>57.9</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F37" s="2">
+        <f t="shared" si="0"/>
+        <v>0.59166666666666667</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1058,13 +1232,17 @@
         <v>1.04</v>
       </c>
       <c r="D38">
-        <v>0.728</v>
+        <v>0.72799999999999998</v>
       </c>
       <c r="E38">
         <v>36</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F38" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1080,8 +1258,12 @@
       <c r="E39">
         <v>57.3</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F39" s="2">
+        <f t="shared" si="0"/>
+        <v>0.70192307692307687</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1092,13 +1274,17 @@
         <v>1.04</v>
       </c>
       <c r="D40">
-        <v>0.736</v>
+        <v>0.73599999999999999</v>
       </c>
       <c r="E40">
         <v>27</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F40" s="2">
+        <f t="shared" si="0"/>
+        <v>0.70769230769230762</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1109,13 +1295,17 @@
         <v>1.04</v>
       </c>
       <c r="D41">
-        <v>0.704</v>
+        <v>0.70399999999999996</v>
       </c>
       <c r="E41">
         <v>47.4</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F41" s="2">
+        <f t="shared" si="0"/>
+        <v>0.67692307692307685</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1126,13 +1316,17 @@
         <v>1.04</v>
       </c>
       <c r="D42">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E42">
         <v>11.3</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F42" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1143,13 +1337,17 @@
         <v>1.04</v>
       </c>
       <c r="D43">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E43">
         <v>36</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F43" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1160,13 +1358,17 @@
         <v>1.04</v>
       </c>
       <c r="D44">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E44">
         <v>19</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F44" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1177,13 +1379,17 @@
         <v>1.04</v>
       </c>
       <c r="D45">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E45">
         <v>20</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F45" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1194,13 +1400,17 @@
         <v>1.04</v>
       </c>
       <c r="D46">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E46">
         <v>15.8</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F46" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1211,13 +1421,17 @@
         <v>1.04</v>
       </c>
       <c r="D47">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E47">
         <v>13.7</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F47" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1228,13 +1442,17 @@
         <v>1.04</v>
       </c>
       <c r="D48">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E48">
         <v>15</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F48" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1245,13 +1463,17 @@
         <v>1.04</v>
       </c>
       <c r="D49">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E49">
         <v>8.5</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F49" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1262,14 +1484,18 @@
         <v>1.04</v>
       </c>
       <c r="D50">
-        <v>0.744</v>
+        <v>0.74399999999999999</v>
       </c>
       <c r="E50">
         <v>12.6</v>
       </c>
+      <c r="F50" s="2">
+        <f t="shared" si="0"/>
+        <v>0.7153846153846154</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>